<commit_message>
feat: fetch_solar_data.py 추가 - 매일 자동 데이터 수집
</commit_message>
<xml_diff>
--- a/train_log.xlsx
+++ b/train_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G721"/>
+  <dimension ref="A1:G745"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1308,7 +1308,7 @@
         <v>7.39</v>
       </c>
       <c r="E33" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F33" t="n">
         <v>9.58</v>
@@ -6357,7 +6357,7 @@
         <v>0</v>
       </c>
       <c r="E220" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F220" t="n">
         <v>0</v>
@@ -12735,7 +12735,7 @@
         <v>0</v>
       </c>
       <c r="G456" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="457">
@@ -12762,7 +12762,7 @@
         <v>0</v>
       </c>
       <c r="G457" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="458">
@@ -19891,6 +19891,654 @@
       </c>
       <c r="G721" t="n">
         <v>1.8</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C722" t="n">
+        <v>0</v>
+      </c>
+      <c r="D722" t="n">
+        <v>0</v>
+      </c>
+      <c r="E722" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="F722" t="n">
+        <v>0</v>
+      </c>
+      <c r="G722" t="n">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C723" t="n">
+        <v>0</v>
+      </c>
+      <c r="D723" t="n">
+        <v>0</v>
+      </c>
+      <c r="E723" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="F723" t="n">
+        <v>0</v>
+      </c>
+      <c r="G723" t="n">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C724" t="n">
+        <v>0</v>
+      </c>
+      <c r="D724" t="n">
+        <v>0</v>
+      </c>
+      <c r="E724" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F724" t="n">
+        <v>0</v>
+      </c>
+      <c r="G724" t="n">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C725" t="n">
+        <v>0</v>
+      </c>
+      <c r="D725" t="n">
+        <v>0</v>
+      </c>
+      <c r="E725" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="F725" t="n">
+        <v>0</v>
+      </c>
+      <c r="G725" t="n">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C726" t="n">
+        <v>0</v>
+      </c>
+      <c r="D726" t="n">
+        <v>0</v>
+      </c>
+      <c r="E726" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F726" t="n">
+        <v>0</v>
+      </c>
+      <c r="G726" t="n">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C727" t="n">
+        <v>0</v>
+      </c>
+      <c r="D727" t="n">
+        <v>0</v>
+      </c>
+      <c r="E727" t="n">
+        <v>10</v>
+      </c>
+      <c r="F727" t="n">
+        <v>0</v>
+      </c>
+      <c r="G727" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C728" t="n">
+        <v>0</v>
+      </c>
+      <c r="D728" t="n">
+        <v>0</v>
+      </c>
+      <c r="E728" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="F728" t="n">
+        <v>0</v>
+      </c>
+      <c r="G728" t="n">
+        <v>9.699999999999999</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C729" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D729" t="n">
+        <v>6</v>
+      </c>
+      <c r="E729" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="F729" t="n">
+        <v>6</v>
+      </c>
+      <c r="G729" t="n">
+        <v>9.800000000000001</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C730" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="D730" t="n">
+        <v>71</v>
+      </c>
+      <c r="E730" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F730" t="n">
+        <v>71</v>
+      </c>
+      <c r="G730" t="n">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C731" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="D731" t="n">
+        <v>164</v>
+      </c>
+      <c r="E731" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="F731" t="n">
+        <v>164</v>
+      </c>
+      <c r="G731" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C732" t="n">
+        <v>34.04</v>
+      </c>
+      <c r="D732" t="n">
+        <v>419</v>
+      </c>
+      <c r="E732" t="n">
+        <v>13</v>
+      </c>
+      <c r="F732" t="n">
+        <v>419</v>
+      </c>
+      <c r="G732" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C733" t="n">
+        <v>19.83</v>
+      </c>
+      <c r="D733" t="n">
+        <v>243</v>
+      </c>
+      <c r="E733" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="F733" t="n">
+        <v>243</v>
+      </c>
+      <c r="G733" t="n">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C734" t="n">
+        <v>14.36</v>
+      </c>
+      <c r="D734" t="n">
+        <v>176</v>
+      </c>
+      <c r="E734" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="F734" t="n">
+        <v>176</v>
+      </c>
+      <c r="G734" t="n">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C735" t="n">
+        <v>19.42</v>
+      </c>
+      <c r="D735" t="n">
+        <v>238</v>
+      </c>
+      <c r="E735" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="F735" t="n">
+        <v>238</v>
+      </c>
+      <c r="G735" t="n">
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C736" t="n">
+        <v>24.89</v>
+      </c>
+      <c r="D736" t="n">
+        <v>305</v>
+      </c>
+      <c r="E736" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="F736" t="n">
+        <v>305</v>
+      </c>
+      <c r="G736" t="n">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C737" t="n">
+        <v>18.93</v>
+      </c>
+      <c r="D737" t="n">
+        <v>232</v>
+      </c>
+      <c r="E737" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="F737" t="n">
+        <v>232</v>
+      </c>
+      <c r="G737" t="n">
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C738" t="n">
+        <v>17.71</v>
+      </c>
+      <c r="D738" t="n">
+        <v>217</v>
+      </c>
+      <c r="E738" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="F738" t="n">
+        <v>217</v>
+      </c>
+      <c r="G738" t="n">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C739" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="D739" t="n">
+        <v>134</v>
+      </c>
+      <c r="E739" t="n">
+        <v>12</v>
+      </c>
+      <c r="F739" t="n">
+        <v>134</v>
+      </c>
+      <c r="G739" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C740" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="D740" t="n">
+        <v>88</v>
+      </c>
+      <c r="E740" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="F740" t="n">
+        <v>88</v>
+      </c>
+      <c r="G740" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C741" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="D741" t="n">
+        <v>17</v>
+      </c>
+      <c r="E741" t="n">
+        <v>10</v>
+      </c>
+      <c r="F741" t="n">
+        <v>17</v>
+      </c>
+      <c r="G741" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C742" t="n">
+        <v>0</v>
+      </c>
+      <c r="D742" t="n">
+        <v>0</v>
+      </c>
+      <c r="E742" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="F742" t="n">
+        <v>0</v>
+      </c>
+      <c r="G742" t="n">
+        <v>9.800000000000001</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C743" t="n">
+        <v>0</v>
+      </c>
+      <c r="D743" t="n">
+        <v>0</v>
+      </c>
+      <c r="E743" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F743" t="n">
+        <v>0</v>
+      </c>
+      <c r="G743" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C744" t="n">
+        <v>0</v>
+      </c>
+      <c r="D744" t="n">
+        <v>0</v>
+      </c>
+      <c r="E744" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="F744" t="n">
+        <v>0</v>
+      </c>
+      <c r="G744" t="n">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C745" t="n">
+        <v>0</v>
+      </c>
+      <c r="D745" t="n">
+        <v>0</v>
+      </c>
+      <c r="E745" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="F745" t="n">
+        <v>0</v>
+      </c>
+      <c r="G745" t="n">
+        <v>8.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: solar data update 2026-08-11
</commit_message>
<xml_diff>
--- a/train_log.xlsx
+++ b/train_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G456"/>
+  <dimension ref="A1:G624"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12738,6 +12738,4542 @@
         <v>28.7</v>
       </c>
     </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C457" t="n">
+        <v>0</v>
+      </c>
+      <c r="D457" t="n">
+        <v>0</v>
+      </c>
+      <c r="E457" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="F457" t="n">
+        <v>0</v>
+      </c>
+      <c r="G457" t="n">
+        <v>27.9</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C458" t="n">
+        <v>0</v>
+      </c>
+      <c r="D458" t="n">
+        <v>0</v>
+      </c>
+      <c r="E458" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="F458" t="n">
+        <v>0</v>
+      </c>
+      <c r="G458" t="n">
+        <v>26.8</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C459" t="n">
+        <v>0</v>
+      </c>
+      <c r="D459" t="n">
+        <v>0</v>
+      </c>
+      <c r="E459" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="F459" t="n">
+        <v>0</v>
+      </c>
+      <c r="G459" t="n">
+        <v>26.1</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C460" t="n">
+        <v>0</v>
+      </c>
+      <c r="D460" t="n">
+        <v>0</v>
+      </c>
+      <c r="E460" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="F460" t="n">
+        <v>0</v>
+      </c>
+      <c r="G460" t="n">
+        <v>25.7</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C461" t="n">
+        <v>0</v>
+      </c>
+      <c r="D461" t="n">
+        <v>0</v>
+      </c>
+      <c r="E461" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="F461" t="n">
+        <v>0</v>
+      </c>
+      <c r="G461" t="n">
+        <v>24.8</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C462" t="n">
+        <v>0</v>
+      </c>
+      <c r="D462" t="n">
+        <v>0</v>
+      </c>
+      <c r="E462" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="F462" t="n">
+        <v>0</v>
+      </c>
+      <c r="G462" t="n">
+        <v>24.3</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C463" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D463" t="n">
+        <v>4</v>
+      </c>
+      <c r="E463" t="n">
+        <v>24</v>
+      </c>
+      <c r="F463" t="n">
+        <v>4</v>
+      </c>
+      <c r="G463" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C464" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="D464" t="n">
+        <v>103</v>
+      </c>
+      <c r="E464" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="F464" t="n">
+        <v>103</v>
+      </c>
+      <c r="G464" t="n">
+        <v>26.3</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C465" t="n">
+        <v>22.46</v>
+      </c>
+      <c r="D465" t="n">
+        <v>290</v>
+      </c>
+      <c r="E465" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="F465" t="n">
+        <v>290</v>
+      </c>
+      <c r="G465" t="n">
+        <v>28.7</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C466" t="n">
+        <v>36.53</v>
+      </c>
+      <c r="D466" t="n">
+        <v>490</v>
+      </c>
+      <c r="E466" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="F466" t="n">
+        <v>490</v>
+      </c>
+      <c r="G466" t="n">
+        <v>31.3</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C467" t="n">
+        <v>48.54</v>
+      </c>
+      <c r="D467" t="n">
+        <v>673</v>
+      </c>
+      <c r="E467" t="n">
+        <v>33</v>
+      </c>
+      <c r="F467" t="n">
+        <v>673</v>
+      </c>
+      <c r="G467" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C468" t="n">
+        <v>57.09</v>
+      </c>
+      <c r="D468" t="n">
+        <v>814</v>
+      </c>
+      <c r="E468" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="F468" t="n">
+        <v>814</v>
+      </c>
+      <c r="G468" t="n">
+        <v>34.7</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C469" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="D469" t="n">
+        <v>907</v>
+      </c>
+      <c r="E469" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="F469" t="n">
+        <v>907</v>
+      </c>
+      <c r="G469" t="n">
+        <v>36.2</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C470" t="n">
+        <v>63.68</v>
+      </c>
+      <c r="D470" t="n">
+        <v>937</v>
+      </c>
+      <c r="E470" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="F470" t="n">
+        <v>937</v>
+      </c>
+      <c r="G470" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C471" t="n">
+        <v>61.86</v>
+      </c>
+      <c r="D471" t="n">
+        <v>911</v>
+      </c>
+      <c r="E471" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="F471" t="n">
+        <v>911</v>
+      </c>
+      <c r="G471" t="n">
+        <v>38.5</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C472" t="n">
+        <v>56.55</v>
+      </c>
+      <c r="D472" t="n">
+        <v>821</v>
+      </c>
+      <c r="E472" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="F472" t="n">
+        <v>821</v>
+      </c>
+      <c r="G472" t="n">
+        <v>38.3</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C473" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="D473" t="n">
+        <v>687</v>
+      </c>
+      <c r="E473" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="F473" t="n">
+        <v>687</v>
+      </c>
+      <c r="G473" t="n">
+        <v>36.8</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C474" t="n">
+        <v>36.91</v>
+      </c>
+      <c r="D474" t="n">
+        <v>506</v>
+      </c>
+      <c r="E474" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="F474" t="n">
+        <v>506</v>
+      </c>
+      <c r="G474" t="n">
+        <v>35.7</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C475" t="n">
+        <v>23.56</v>
+      </c>
+      <c r="D475" t="n">
+        <v>312</v>
+      </c>
+      <c r="E475" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="F475" t="n">
+        <v>312</v>
+      </c>
+      <c r="G475" t="n">
+        <v>33.9</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C476" t="n">
+        <v>9.44</v>
+      </c>
+      <c r="D476" t="n">
+        <v>121</v>
+      </c>
+      <c r="E476" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="F476" t="n">
+        <v>121</v>
+      </c>
+      <c r="G476" t="n">
+        <v>32.3</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C477" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="D477" t="n">
+        <v>8</v>
+      </c>
+      <c r="E477" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="F477" t="n">
+        <v>8</v>
+      </c>
+      <c r="G477" t="n">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C478" t="n">
+        <v>0</v>
+      </c>
+      <c r="D478" t="n">
+        <v>0</v>
+      </c>
+      <c r="E478" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="F478" t="n">
+        <v>0</v>
+      </c>
+      <c r="G478" t="n">
+        <v>31.6</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C479" t="n">
+        <v>0</v>
+      </c>
+      <c r="D479" t="n">
+        <v>0</v>
+      </c>
+      <c r="E479" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="F479" t="n">
+        <v>0</v>
+      </c>
+      <c r="G479" t="n">
+        <v>30.7</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C480" t="n">
+        <v>0</v>
+      </c>
+      <c r="D480" t="n">
+        <v>0</v>
+      </c>
+      <c r="E480" t="n">
+        <v>30</v>
+      </c>
+      <c r="F480" t="n">
+        <v>0</v>
+      </c>
+      <c r="G480" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C481" t="n">
+        <v>0</v>
+      </c>
+      <c r="D481" t="n">
+        <v>0</v>
+      </c>
+      <c r="E481" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="F481" t="n">
+        <v>0</v>
+      </c>
+      <c r="G481" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C482" t="n">
+        <v>0</v>
+      </c>
+      <c r="D482" t="n">
+        <v>0</v>
+      </c>
+      <c r="E482" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="F482" t="n">
+        <v>0</v>
+      </c>
+      <c r="G482" t="n">
+        <v>27.9</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C483" t="n">
+        <v>0</v>
+      </c>
+      <c r="D483" t="n">
+        <v>0</v>
+      </c>
+      <c r="E483" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="F483" t="n">
+        <v>0</v>
+      </c>
+      <c r="G483" t="n">
+        <v>27.4</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C484" t="n">
+        <v>0</v>
+      </c>
+      <c r="D484" t="n">
+        <v>0</v>
+      </c>
+      <c r="E484" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="F484" t="n">
+        <v>0</v>
+      </c>
+      <c r="G484" t="n">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>0</v>
+      </c>
+      <c r="D485" t="n">
+        <v>0</v>
+      </c>
+      <c r="E485" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="F485" t="n">
+        <v>0</v>
+      </c>
+      <c r="G485" t="n">
+        <v>26.8</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>0</v>
+      </c>
+      <c r="D486" t="n">
+        <v>0</v>
+      </c>
+      <c r="E486" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="F486" t="n">
+        <v>0</v>
+      </c>
+      <c r="G486" t="n">
+        <v>26.2</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D487" t="n">
+        <v>3</v>
+      </c>
+      <c r="E487" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="F487" t="n">
+        <v>3</v>
+      </c>
+      <c r="G487" t="n">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C488" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="D488" t="n">
+        <v>99</v>
+      </c>
+      <c r="E488" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="F488" t="n">
+        <v>99</v>
+      </c>
+      <c r="G488" t="n">
+        <v>28.2</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C489" t="n">
+        <v>21.78</v>
+      </c>
+      <c r="D489" t="n">
+        <v>283</v>
+      </c>
+      <c r="E489" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="F489" t="n">
+        <v>283</v>
+      </c>
+      <c r="G489" t="n">
+        <v>30.4</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C490" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="D490" t="n">
+        <v>481</v>
+      </c>
+      <c r="E490" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="F490" t="n">
+        <v>481</v>
+      </c>
+      <c r="G490" t="n">
+        <v>32.6</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C491" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="D491" t="n">
+        <v>661</v>
+      </c>
+      <c r="E491" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="F491" t="n">
+        <v>661</v>
+      </c>
+      <c r="G491" t="n">
+        <v>33.7</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C492" t="n">
+        <v>56.35</v>
+      </c>
+      <c r="D492" t="n">
+        <v>803</v>
+      </c>
+      <c r="E492" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="F492" t="n">
+        <v>803</v>
+      </c>
+      <c r="G492" t="n">
+        <v>34.9</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C493" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="D493" t="n">
+        <v>892</v>
+      </c>
+      <c r="E493" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="F493" t="n">
+        <v>892</v>
+      </c>
+      <c r="G493" t="n">
+        <v>35.8</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C494" t="n">
+        <v>61.92</v>
+      </c>
+      <c r="D494" t="n">
+        <v>898</v>
+      </c>
+      <c r="E494" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="F494" t="n">
+        <v>898</v>
+      </c>
+      <c r="G494" t="n">
+        <v>35.7</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C495" t="n">
+        <v>60.82</v>
+      </c>
+      <c r="D495" t="n">
+        <v>875</v>
+      </c>
+      <c r="E495" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="F495" t="n">
+        <v>875</v>
+      </c>
+      <c r="G495" t="n">
+        <v>34.7</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C496" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="D496" t="n">
+        <v>788</v>
+      </c>
+      <c r="E496" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="F496" t="n">
+        <v>788</v>
+      </c>
+      <c r="G496" t="n">
+        <v>34.6</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C497" t="n">
+        <v>45.94</v>
+      </c>
+      <c r="D497" t="n">
+        <v>634</v>
+      </c>
+      <c r="E497" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="F497" t="n">
+        <v>634</v>
+      </c>
+      <c r="G497" t="n">
+        <v>33.2</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C498" t="n">
+        <v>32.85</v>
+      </c>
+      <c r="D498" t="n">
+        <v>439</v>
+      </c>
+      <c r="E498" t="n">
+        <v>32</v>
+      </c>
+      <c r="F498" t="n">
+        <v>439</v>
+      </c>
+      <c r="G498" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C499" t="n">
+        <v>22.27</v>
+      </c>
+      <c r="D499" t="n">
+        <v>289</v>
+      </c>
+      <c r="E499" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="F499" t="n">
+        <v>289</v>
+      </c>
+      <c r="G499" t="n">
+        <v>29.9</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C500" t="n">
+        <v>9.029999999999999</v>
+      </c>
+      <c r="D500" t="n">
+        <v>114</v>
+      </c>
+      <c r="E500" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="F500" t="n">
+        <v>114</v>
+      </c>
+      <c r="G500" t="n">
+        <v>28.7</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C501" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D501" t="n">
+        <v>7</v>
+      </c>
+      <c r="E501" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="F501" t="n">
+        <v>7</v>
+      </c>
+      <c r="G501" t="n">
+        <v>28.2</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C502" t="n">
+        <v>0</v>
+      </c>
+      <c r="D502" t="n">
+        <v>0</v>
+      </c>
+      <c r="E502" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="F502" t="n">
+        <v>0</v>
+      </c>
+      <c r="G502" t="n">
+        <v>28.6</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C503" t="n">
+        <v>0</v>
+      </c>
+      <c r="D503" t="n">
+        <v>0</v>
+      </c>
+      <c r="E503" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="F503" t="n">
+        <v>0</v>
+      </c>
+      <c r="G503" t="n">
+        <v>27.9</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C504" t="n">
+        <v>0</v>
+      </c>
+      <c r="D504" t="n">
+        <v>0</v>
+      </c>
+      <c r="E504" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="F504" t="n">
+        <v>0</v>
+      </c>
+      <c r="G504" t="n">
+        <v>27.4</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C505" t="n">
+        <v>0</v>
+      </c>
+      <c r="D505" t="n">
+        <v>0</v>
+      </c>
+      <c r="E505" t="n">
+        <v>27</v>
+      </c>
+      <c r="F505" t="n">
+        <v>0</v>
+      </c>
+      <c r="G505" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C506" t="n">
+        <v>0</v>
+      </c>
+      <c r="D506" t="n">
+        <v>0</v>
+      </c>
+      <c r="E506" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="F506" t="n">
+        <v>0</v>
+      </c>
+      <c r="G506" t="n">
+        <v>26.7</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C507" t="n">
+        <v>0</v>
+      </c>
+      <c r="D507" t="n">
+        <v>0</v>
+      </c>
+      <c r="E507" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="F507" t="n">
+        <v>0</v>
+      </c>
+      <c r="G507" t="n">
+        <v>26.3</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C508" t="n">
+        <v>0</v>
+      </c>
+      <c r="D508" t="n">
+        <v>0</v>
+      </c>
+      <c r="E508" t="n">
+        <v>26</v>
+      </c>
+      <c r="F508" t="n">
+        <v>0</v>
+      </c>
+      <c r="G508" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C509" t="n">
+        <v>0</v>
+      </c>
+      <c r="D509" t="n">
+        <v>0</v>
+      </c>
+      <c r="E509" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="F509" t="n">
+        <v>0</v>
+      </c>
+      <c r="G509" t="n">
+        <v>25.3</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C510" t="n">
+        <v>0</v>
+      </c>
+      <c r="D510" t="n">
+        <v>0</v>
+      </c>
+      <c r="E510" t="n">
+        <v>25</v>
+      </c>
+      <c r="F510" t="n">
+        <v>0</v>
+      </c>
+      <c r="G510" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C511" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D511" t="n">
+        <v>3</v>
+      </c>
+      <c r="E511" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="F511" t="n">
+        <v>3</v>
+      </c>
+      <c r="G511" t="n">
+        <v>24.9</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C512" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="D512" t="n">
+        <v>89</v>
+      </c>
+      <c r="E512" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="F512" t="n">
+        <v>89</v>
+      </c>
+      <c r="G512" t="n">
+        <v>26.7</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C513" t="n">
+        <v>20.81</v>
+      </c>
+      <c r="D513" t="n">
+        <v>268</v>
+      </c>
+      <c r="E513" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="F513" t="n">
+        <v>268</v>
+      </c>
+      <c r="G513" t="n">
+        <v>28.7</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C514" t="n">
+        <v>34.63</v>
+      </c>
+      <c r="D514" t="n">
+        <v>463</v>
+      </c>
+      <c r="E514" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="F514" t="n">
+        <v>463</v>
+      </c>
+      <c r="G514" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C515" t="n">
+        <v>44.37</v>
+      </c>
+      <c r="D515" t="n">
+        <v>608</v>
+      </c>
+      <c r="E515" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="F515" t="n">
+        <v>608</v>
+      </c>
+      <c r="G515" t="n">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C516" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="D516" t="n">
+        <v>724</v>
+      </c>
+      <c r="E516" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="F516" t="n">
+        <v>724</v>
+      </c>
+      <c r="G516" t="n">
+        <v>33.6</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C517" t="n">
+        <v>55.87</v>
+      </c>
+      <c r="D517" t="n">
+        <v>794</v>
+      </c>
+      <c r="E517" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="F517" t="n">
+        <v>794</v>
+      </c>
+      <c r="G517" t="n">
+        <v>34.6</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C518" t="n">
+        <v>58.52</v>
+      </c>
+      <c r="D518" t="n">
+        <v>835</v>
+      </c>
+      <c r="E518" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="F518" t="n">
+        <v>835</v>
+      </c>
+      <c r="G518" t="n">
+        <v>34.2</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C519" t="n">
+        <v>56.41</v>
+      </c>
+      <c r="D519" t="n">
+        <v>787</v>
+      </c>
+      <c r="E519" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="F519" t="n">
+        <v>787</v>
+      </c>
+      <c r="G519" t="n">
+        <v>30.8</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C520" t="n">
+        <v>52.17</v>
+      </c>
+      <c r="D520" t="n">
+        <v>720</v>
+      </c>
+      <c r="E520" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="F520" t="n">
+        <v>720</v>
+      </c>
+      <c r="G520" t="n">
+        <v>30.5</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C521" t="n">
+        <v>43.68</v>
+      </c>
+      <c r="D521" t="n">
+        <v>591</v>
+      </c>
+      <c r="E521" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="F521" t="n">
+        <v>591</v>
+      </c>
+      <c r="G521" t="n">
+        <v>30.1</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C522" t="n">
+        <v>34.59</v>
+      </c>
+      <c r="D522" t="n">
+        <v>461</v>
+      </c>
+      <c r="E522" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="F522" t="n">
+        <v>461</v>
+      </c>
+      <c r="G522" t="n">
+        <v>30.7</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C523" t="n">
+        <v>20.19</v>
+      </c>
+      <c r="D523" t="n">
+        <v>261</v>
+      </c>
+      <c r="E523" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="F523" t="n">
+        <v>261</v>
+      </c>
+      <c r="G523" t="n">
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C524" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="D524" t="n">
+        <v>102</v>
+      </c>
+      <c r="E524" t="n">
+        <v>29</v>
+      </c>
+      <c r="F524" t="n">
+        <v>102</v>
+      </c>
+      <c r="G524" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C525" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D525" t="n">
+        <v>5</v>
+      </c>
+      <c r="E525" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="F525" t="n">
+        <v>5</v>
+      </c>
+      <c r="G525" t="n">
+        <v>27.9</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C526" t="n">
+        <v>0</v>
+      </c>
+      <c r="D526" t="n">
+        <v>0</v>
+      </c>
+      <c r="E526" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="F526" t="n">
+        <v>0</v>
+      </c>
+      <c r="G526" t="n">
+        <v>28.4</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C527" t="n">
+        <v>0</v>
+      </c>
+      <c r="D527" t="n">
+        <v>0</v>
+      </c>
+      <c r="E527" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="F527" t="n">
+        <v>0</v>
+      </c>
+      <c r="G527" t="n">
+        <v>27.6</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C528" t="n">
+        <v>0</v>
+      </c>
+      <c r="D528" t="n">
+        <v>0</v>
+      </c>
+      <c r="E528" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="F528" t="n">
+        <v>0</v>
+      </c>
+      <c r="G528" t="n">
+        <v>26.6</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C529" t="n">
+        <v>0</v>
+      </c>
+      <c r="D529" t="n">
+        <v>0</v>
+      </c>
+      <c r="E529" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="F529" t="n">
+        <v>0</v>
+      </c>
+      <c r="G529" t="n">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C530" t="n">
+        <v>0</v>
+      </c>
+      <c r="D530" t="n">
+        <v>0</v>
+      </c>
+      <c r="E530" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="F530" t="n">
+        <v>0</v>
+      </c>
+      <c r="G530" t="n">
+        <v>25.7</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C531" t="n">
+        <v>0</v>
+      </c>
+      <c r="D531" t="n">
+        <v>0</v>
+      </c>
+      <c r="E531" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F531" t="n">
+        <v>0</v>
+      </c>
+      <c r="G531" t="n">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C532" t="n">
+        <v>0</v>
+      </c>
+      <c r="D532" t="n">
+        <v>0</v>
+      </c>
+      <c r="E532" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="F532" t="n">
+        <v>0</v>
+      </c>
+      <c r="G532" t="n">
+        <v>25.4</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C533" t="n">
+        <v>0</v>
+      </c>
+      <c r="D533" t="n">
+        <v>0</v>
+      </c>
+      <c r="E533" t="n">
+        <v>25</v>
+      </c>
+      <c r="F533" t="n">
+        <v>0</v>
+      </c>
+      <c r="G533" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C534" t="n">
+        <v>0</v>
+      </c>
+      <c r="D534" t="n">
+        <v>0</v>
+      </c>
+      <c r="E534" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="F534" t="n">
+        <v>0</v>
+      </c>
+      <c r="G534" t="n">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C535" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D535" t="n">
+        <v>2</v>
+      </c>
+      <c r="E535" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="F535" t="n">
+        <v>2</v>
+      </c>
+      <c r="G535" t="n">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C536" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="D536" t="n">
+        <v>87</v>
+      </c>
+      <c r="E536" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="F536" t="n">
+        <v>87</v>
+      </c>
+      <c r="G536" t="n">
+        <v>26.1</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C537" t="n">
+        <v>19.92</v>
+      </c>
+      <c r="D537" t="n">
+        <v>255</v>
+      </c>
+      <c r="E537" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="F537" t="n">
+        <v>255</v>
+      </c>
+      <c r="G537" t="n">
+        <v>27.7</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C538" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="D538" t="n">
+        <v>434</v>
+      </c>
+      <c r="E538" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="F538" t="n">
+        <v>434</v>
+      </c>
+      <c r="G538" t="n">
+        <v>30.2</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C539" t="n">
+        <v>44.28</v>
+      </c>
+      <c r="D539" t="n">
+        <v>603</v>
+      </c>
+      <c r="E539" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="F539" t="n">
+        <v>603</v>
+      </c>
+      <c r="G539" t="n">
+        <v>31.2</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C540" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="D540" t="n">
+        <v>724</v>
+      </c>
+      <c r="E540" t="n">
+        <v>32</v>
+      </c>
+      <c r="F540" t="n">
+        <v>724</v>
+      </c>
+      <c r="G540" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C541" t="n">
+        <v>57.87</v>
+      </c>
+      <c r="D541" t="n">
+        <v>818</v>
+      </c>
+      <c r="E541" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="F541" t="n">
+        <v>818</v>
+      </c>
+      <c r="G541" t="n">
+        <v>32.7</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C542" t="n">
+        <v>60.54</v>
+      </c>
+      <c r="D542" t="n">
+        <v>858</v>
+      </c>
+      <c r="E542" t="n">
+        <v>32</v>
+      </c>
+      <c r="F542" t="n">
+        <v>858</v>
+      </c>
+      <c r="G542" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C543" t="n">
+        <v>59.77</v>
+      </c>
+      <c r="D543" t="n">
+        <v>845</v>
+      </c>
+      <c r="E543" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="F543" t="n">
+        <v>845</v>
+      </c>
+      <c r="G543" t="n">
+        <v>31.9</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C544" t="n">
+        <v>53.68</v>
+      </c>
+      <c r="D544" t="n">
+        <v>750</v>
+      </c>
+      <c r="E544" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="F544" t="n">
+        <v>750</v>
+      </c>
+      <c r="G544" t="n">
+        <v>32.3</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C545" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="D545" t="n">
+        <v>604</v>
+      </c>
+      <c r="E545" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="F545" t="n">
+        <v>604</v>
+      </c>
+      <c r="G545" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C546" t="n">
+        <v>34.53</v>
+      </c>
+      <c r="D546" t="n">
+        <v>459</v>
+      </c>
+      <c r="E546" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="F546" t="n">
+        <v>459</v>
+      </c>
+      <c r="G546" t="n">
+        <v>30.2</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C547" t="n">
+        <v>21.45</v>
+      </c>
+      <c r="D547" t="n">
+        <v>277</v>
+      </c>
+      <c r="E547" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="F547" t="n">
+        <v>277</v>
+      </c>
+      <c r="G547" t="n">
+        <v>29.1</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C548" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="D548" t="n">
+        <v>107</v>
+      </c>
+      <c r="E548" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="F548" t="n">
+        <v>107</v>
+      </c>
+      <c r="G548" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C549" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D549" t="n">
+        <v>6</v>
+      </c>
+      <c r="E549" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="F549" t="n">
+        <v>6</v>
+      </c>
+      <c r="G549" t="n">
+        <v>27.3</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C550" t="n">
+        <v>0</v>
+      </c>
+      <c r="D550" t="n">
+        <v>0</v>
+      </c>
+      <c r="E550" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="F550" t="n">
+        <v>0</v>
+      </c>
+      <c r="G550" t="n">
+        <v>26.9</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C551" t="n">
+        <v>0</v>
+      </c>
+      <c r="D551" t="n">
+        <v>0</v>
+      </c>
+      <c r="E551" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="F551" t="n">
+        <v>0</v>
+      </c>
+      <c r="G551" t="n">
+        <v>26.2</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C552" t="n">
+        <v>0</v>
+      </c>
+      <c r="D552" t="n">
+        <v>0</v>
+      </c>
+      <c r="E552" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="F552" t="n">
+        <v>0</v>
+      </c>
+      <c r="G552" t="n">
+        <v>25.7</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C553" t="n">
+        <v>0</v>
+      </c>
+      <c r="D553" t="n">
+        <v>0</v>
+      </c>
+      <c r="E553" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="F553" t="n">
+        <v>0</v>
+      </c>
+      <c r="G553" t="n">
+        <v>25.4</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C554" t="n">
+        <v>0</v>
+      </c>
+      <c r="D554" t="n">
+        <v>0</v>
+      </c>
+      <c r="E554" t="n">
+        <v>25</v>
+      </c>
+      <c r="F554" t="n">
+        <v>0</v>
+      </c>
+      <c r="G554" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C555" t="n">
+        <v>0</v>
+      </c>
+      <c r="D555" t="n">
+        <v>0</v>
+      </c>
+      <c r="E555" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="F555" t="n">
+        <v>0</v>
+      </c>
+      <c r="G555" t="n">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C556" t="n">
+        <v>0</v>
+      </c>
+      <c r="D556" t="n">
+        <v>0</v>
+      </c>
+      <c r="E556" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="F556" t="n">
+        <v>0</v>
+      </c>
+      <c r="G556" t="n">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C557" t="n">
+        <v>0</v>
+      </c>
+      <c r="D557" t="n">
+        <v>0</v>
+      </c>
+      <c r="E557" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="F557" t="n">
+        <v>0</v>
+      </c>
+      <c r="G557" t="n">
+        <v>24.4</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C558" t="n">
+        <v>0</v>
+      </c>
+      <c r="D558" t="n">
+        <v>0</v>
+      </c>
+      <c r="E558" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="F558" t="n">
+        <v>0</v>
+      </c>
+      <c r="G558" t="n">
+        <v>24.4</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C559" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D559" t="n">
+        <v>2</v>
+      </c>
+      <c r="E559" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="F559" t="n">
+        <v>2</v>
+      </c>
+      <c r="G559" t="n">
+        <v>24.3</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C560" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="D560" t="n">
+        <v>90</v>
+      </c>
+      <c r="E560" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="F560" t="n">
+        <v>90</v>
+      </c>
+      <c r="G560" t="n">
+        <v>25.4</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C561" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="D561" t="n">
+        <v>272</v>
+      </c>
+      <c r="E561" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="F561" t="n">
+        <v>272</v>
+      </c>
+      <c r="G561" t="n">
+        <v>27.2</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C562" t="n">
+        <v>35.45</v>
+      </c>
+      <c r="D562" t="n">
+        <v>471</v>
+      </c>
+      <c r="E562" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="F562" t="n">
+        <v>471</v>
+      </c>
+      <c r="G562" t="n">
+        <v>29.7</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C563" t="n">
+        <v>47.57</v>
+      </c>
+      <c r="D563" t="n">
+        <v>652</v>
+      </c>
+      <c r="E563" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="F563" t="n">
+        <v>652</v>
+      </c>
+      <c r="G563" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C564" t="n">
+        <v>56.29</v>
+      </c>
+      <c r="D564" t="n">
+        <v>794</v>
+      </c>
+      <c r="E564" t="n">
+        <v>33</v>
+      </c>
+      <c r="F564" t="n">
+        <v>794</v>
+      </c>
+      <c r="G564" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C565" t="n">
+        <v>61.09</v>
+      </c>
+      <c r="D565" t="n">
+        <v>879</v>
+      </c>
+      <c r="E565" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="F565" t="n">
+        <v>879</v>
+      </c>
+      <c r="G565" t="n">
+        <v>34.6</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C566" t="n">
+        <v>57.51</v>
+      </c>
+      <c r="D566" t="n">
+        <v>817</v>
+      </c>
+      <c r="E566" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="F566" t="n">
+        <v>817</v>
+      </c>
+      <c r="G566" t="n">
+        <v>33.8</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C567" t="n">
+        <v>55.81</v>
+      </c>
+      <c r="D567" t="n">
+        <v>791</v>
+      </c>
+      <c r="E567" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="F567" t="n">
+        <v>791</v>
+      </c>
+      <c r="G567" t="n">
+        <v>34.1</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C568" t="n">
+        <v>55.47</v>
+      </c>
+      <c r="D568" t="n">
+        <v>781</v>
+      </c>
+      <c r="E568" t="n">
+        <v>33</v>
+      </c>
+      <c r="F568" t="n">
+        <v>781</v>
+      </c>
+      <c r="G568" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C569" t="n">
+        <v>46.81</v>
+      </c>
+      <c r="D569" t="n">
+        <v>645</v>
+      </c>
+      <c r="E569" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="F569" t="n">
+        <v>645</v>
+      </c>
+      <c r="G569" t="n">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C570" t="n">
+        <v>37.16</v>
+      </c>
+      <c r="D570" t="n">
+        <v>501</v>
+      </c>
+      <c r="E570" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="F570" t="n">
+        <v>501</v>
+      </c>
+      <c r="G570" t="n">
+        <v>32.1</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C571" t="n">
+        <v>22.95</v>
+      </c>
+      <c r="D571" t="n">
+        <v>300</v>
+      </c>
+      <c r="E571" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="F571" t="n">
+        <v>300</v>
+      </c>
+      <c r="G571" t="n">
+        <v>31.2</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C572" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="D572" t="n">
+        <v>112</v>
+      </c>
+      <c r="E572" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="F572" t="n">
+        <v>112</v>
+      </c>
+      <c r="G572" t="n">
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C573" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D573" t="n">
+        <v>6</v>
+      </c>
+      <c r="E573" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="F573" t="n">
+        <v>6</v>
+      </c>
+      <c r="G573" t="n">
+        <v>28.3</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C574" t="n">
+        <v>0</v>
+      </c>
+      <c r="D574" t="n">
+        <v>0</v>
+      </c>
+      <c r="E574" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="F574" t="n">
+        <v>0</v>
+      </c>
+      <c r="G574" t="n">
+        <v>28.3</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C575" t="n">
+        <v>0</v>
+      </c>
+      <c r="D575" t="n">
+        <v>0</v>
+      </c>
+      <c r="E575" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="F575" t="n">
+        <v>0</v>
+      </c>
+      <c r="G575" t="n">
+        <v>27.4</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C576" t="n">
+        <v>0</v>
+      </c>
+      <c r="D576" t="n">
+        <v>0</v>
+      </c>
+      <c r="E576" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="F576" t="n">
+        <v>0</v>
+      </c>
+      <c r="G576" t="n">
+        <v>26.6</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C577" t="n">
+        <v>0</v>
+      </c>
+      <c r="D577" t="n">
+        <v>0</v>
+      </c>
+      <c r="E577" t="n">
+        <v>0</v>
+      </c>
+      <c r="F577" t="n">
+        <v>0</v>
+      </c>
+      <c r="G577" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C578" t="n">
+        <v>0</v>
+      </c>
+      <c r="D578" t="n">
+        <v>0</v>
+      </c>
+      <c r="E578" t="n">
+        <v>0</v>
+      </c>
+      <c r="F578" t="n">
+        <v>0</v>
+      </c>
+      <c r="G578" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C579" t="n">
+        <v>0</v>
+      </c>
+      <c r="D579" t="n">
+        <v>0</v>
+      </c>
+      <c r="E579" t="n">
+        <v>0</v>
+      </c>
+      <c r="F579" t="n">
+        <v>0</v>
+      </c>
+      <c r="G579" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C580" t="n">
+        <v>0</v>
+      </c>
+      <c r="D580" t="n">
+        <v>0</v>
+      </c>
+      <c r="E580" t="n">
+        <v>0</v>
+      </c>
+      <c r="F580" t="n">
+        <v>0</v>
+      </c>
+      <c r="G580" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C581" t="n">
+        <v>0</v>
+      </c>
+      <c r="D581" t="n">
+        <v>0</v>
+      </c>
+      <c r="E581" t="n">
+        <v>0</v>
+      </c>
+      <c r="F581" t="n">
+        <v>0</v>
+      </c>
+      <c r="G581" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C582" t="n">
+        <v>0</v>
+      </c>
+      <c r="D582" t="n">
+        <v>0</v>
+      </c>
+      <c r="E582" t="n">
+        <v>0</v>
+      </c>
+      <c r="F582" t="n">
+        <v>0</v>
+      </c>
+      <c r="G582" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C583" t="n">
+        <v>0</v>
+      </c>
+      <c r="D583" t="n">
+        <v>0</v>
+      </c>
+      <c r="E583" t="n">
+        <v>0</v>
+      </c>
+      <c r="F583" t="n">
+        <v>0</v>
+      </c>
+      <c r="G583" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C584" t="n">
+        <v>0</v>
+      </c>
+      <c r="D584" t="n">
+        <v>0</v>
+      </c>
+      <c r="E584" t="n">
+        <v>0</v>
+      </c>
+      <c r="F584" t="n">
+        <v>0</v>
+      </c>
+      <c r="G584" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C585" t="n">
+        <v>0</v>
+      </c>
+      <c r="D585" t="n">
+        <v>0</v>
+      </c>
+      <c r="E585" t="n">
+        <v>0</v>
+      </c>
+      <c r="F585" t="n">
+        <v>0</v>
+      </c>
+      <c r="G585" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C586" t="n">
+        <v>0</v>
+      </c>
+      <c r="D586" t="n">
+        <v>0</v>
+      </c>
+      <c r="E586" t="n">
+        <v>0</v>
+      </c>
+      <c r="F586" t="n">
+        <v>0</v>
+      </c>
+      <c r="G586" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C587" t="n">
+        <v>0</v>
+      </c>
+      <c r="D587" t="n">
+        <v>0</v>
+      </c>
+      <c r="E587" t="n">
+        <v>0</v>
+      </c>
+      <c r="F587" t="n">
+        <v>0</v>
+      </c>
+      <c r="G587" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C588" t="n">
+        <v>0</v>
+      </c>
+      <c r="D588" t="n">
+        <v>0</v>
+      </c>
+      <c r="E588" t="n">
+        <v>0</v>
+      </c>
+      <c r="F588" t="n">
+        <v>0</v>
+      </c>
+      <c r="G588" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C589" t="n">
+        <v>0</v>
+      </c>
+      <c r="D589" t="n">
+        <v>0</v>
+      </c>
+      <c r="E589" t="n">
+        <v>0</v>
+      </c>
+      <c r="F589" t="n">
+        <v>0</v>
+      </c>
+      <c r="G589" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C590" t="n">
+        <v>0</v>
+      </c>
+      <c r="D590" t="n">
+        <v>0</v>
+      </c>
+      <c r="E590" t="n">
+        <v>0</v>
+      </c>
+      <c r="F590" t="n">
+        <v>0</v>
+      </c>
+      <c r="G590" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C591" t="n">
+        <v>0</v>
+      </c>
+      <c r="D591" t="n">
+        <v>0</v>
+      </c>
+      <c r="E591" t="n">
+        <v>0</v>
+      </c>
+      <c r="F591" t="n">
+        <v>0</v>
+      </c>
+      <c r="G591" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C592" t="n">
+        <v>0</v>
+      </c>
+      <c r="D592" t="n">
+        <v>0</v>
+      </c>
+      <c r="E592" t="n">
+        <v>0</v>
+      </c>
+      <c r="F592" t="n">
+        <v>0</v>
+      </c>
+      <c r="G592" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C593" t="n">
+        <v>0</v>
+      </c>
+      <c r="D593" t="n">
+        <v>0</v>
+      </c>
+      <c r="E593" t="n">
+        <v>0</v>
+      </c>
+      <c r="F593" t="n">
+        <v>0</v>
+      </c>
+      <c r="G593" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C594" t="n">
+        <v>0</v>
+      </c>
+      <c r="D594" t="n">
+        <v>0</v>
+      </c>
+      <c r="E594" t="n">
+        <v>0</v>
+      </c>
+      <c r="F594" t="n">
+        <v>0</v>
+      </c>
+      <c r="G594" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C595" t="n">
+        <v>0</v>
+      </c>
+      <c r="D595" t="n">
+        <v>0</v>
+      </c>
+      <c r="E595" t="n">
+        <v>0</v>
+      </c>
+      <c r="F595" t="n">
+        <v>0</v>
+      </c>
+      <c r="G595" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C596" t="n">
+        <v>0</v>
+      </c>
+      <c r="D596" t="n">
+        <v>0</v>
+      </c>
+      <c r="E596" t="n">
+        <v>0</v>
+      </c>
+      <c r="F596" t="n">
+        <v>0</v>
+      </c>
+      <c r="G596" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C597" t="n">
+        <v>0</v>
+      </c>
+      <c r="D597" t="n">
+        <v>0</v>
+      </c>
+      <c r="E597" t="n">
+        <v>0</v>
+      </c>
+      <c r="F597" t="n">
+        <v>0</v>
+      </c>
+      <c r="G597" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C598" t="n">
+        <v>0</v>
+      </c>
+      <c r="D598" t="n">
+        <v>0</v>
+      </c>
+      <c r="E598" t="n">
+        <v>0</v>
+      </c>
+      <c r="F598" t="n">
+        <v>0</v>
+      </c>
+      <c r="G598" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C599" t="n">
+        <v>0</v>
+      </c>
+      <c r="D599" t="n">
+        <v>0</v>
+      </c>
+      <c r="E599" t="n">
+        <v>0</v>
+      </c>
+      <c r="F599" t="n">
+        <v>0</v>
+      </c>
+      <c r="G599" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C600" t="n">
+        <v>0</v>
+      </c>
+      <c r="D600" t="n">
+        <v>0</v>
+      </c>
+      <c r="E600" t="n">
+        <v>0</v>
+      </c>
+      <c r="F600" t="n">
+        <v>0</v>
+      </c>
+      <c r="G600" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>0시</t>
+        </is>
+      </c>
+      <c r="C601" t="n">
+        <v>0</v>
+      </c>
+      <c r="D601" t="n">
+        <v>0</v>
+      </c>
+      <c r="E601" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="F601" t="n">
+        <v>0</v>
+      </c>
+      <c r="G601" t="n">
+        <v>23.6</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>1시</t>
+        </is>
+      </c>
+      <c r="C602" t="n">
+        <v>0</v>
+      </c>
+      <c r="D602" t="n">
+        <v>0</v>
+      </c>
+      <c r="E602" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="F602" t="n">
+        <v>0</v>
+      </c>
+      <c r="G602" t="n">
+        <v>23.9</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>2시</t>
+        </is>
+      </c>
+      <c r="C603" t="n">
+        <v>0</v>
+      </c>
+      <c r="D603" t="n">
+        <v>0</v>
+      </c>
+      <c r="E603" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="F603" t="n">
+        <v>0</v>
+      </c>
+      <c r="G603" t="n">
+        <v>23.2</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>3시</t>
+        </is>
+      </c>
+      <c r="C604" t="n">
+        <v>0</v>
+      </c>
+      <c r="D604" t="n">
+        <v>0</v>
+      </c>
+      <c r="E604" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="F604" t="n">
+        <v>0</v>
+      </c>
+      <c r="G604" t="n">
+        <v>23.2</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>4시</t>
+        </is>
+      </c>
+      <c r="C605" t="n">
+        <v>0</v>
+      </c>
+      <c r="D605" t="n">
+        <v>0</v>
+      </c>
+      <c r="E605" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="F605" t="n">
+        <v>0</v>
+      </c>
+      <c r="G605" t="n">
+        <v>22.9</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>5시</t>
+        </is>
+      </c>
+      <c r="C606" t="n">
+        <v>0</v>
+      </c>
+      <c r="D606" t="n">
+        <v>0</v>
+      </c>
+      <c r="E606" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="F606" t="n">
+        <v>0</v>
+      </c>
+      <c r="G606" t="n">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>6시</t>
+        </is>
+      </c>
+      <c r="C607" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D607" t="n">
+        <v>1</v>
+      </c>
+      <c r="E607" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="F607" t="n">
+        <v>1</v>
+      </c>
+      <c r="G607" t="n">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>7시</t>
+        </is>
+      </c>
+      <c r="C608" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="D608" t="n">
+        <v>30</v>
+      </c>
+      <c r="E608" t="n">
+        <v>23</v>
+      </c>
+      <c r="F608" t="n">
+        <v>30</v>
+      </c>
+      <c r="G608" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>8시</t>
+        </is>
+      </c>
+      <c r="C609" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="D609" t="n">
+        <v>79</v>
+      </c>
+      <c r="E609" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="F609" t="n">
+        <v>79</v>
+      </c>
+      <c r="G609" t="n">
+        <v>23.2</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>9시</t>
+        </is>
+      </c>
+      <c r="C610" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="D610" t="n">
+        <v>189</v>
+      </c>
+      <c r="E610" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="F610" t="n">
+        <v>189</v>
+      </c>
+      <c r="G610" t="n">
+        <v>26.4</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>10시</t>
+        </is>
+      </c>
+      <c r="C611" t="n">
+        <v>28</v>
+      </c>
+      <c r="D611" t="n">
+        <v>363</v>
+      </c>
+      <c r="E611" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="F611" t="n">
+        <v>363</v>
+      </c>
+      <c r="G611" t="n">
+        <v>27.3</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>11시</t>
+        </is>
+      </c>
+      <c r="C612" t="n">
+        <v>38.94</v>
+      </c>
+      <c r="D612" t="n">
+        <v>519</v>
+      </c>
+      <c r="E612" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="F612" t="n">
+        <v>519</v>
+      </c>
+      <c r="G612" t="n">
+        <v>28.9</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>12시</t>
+        </is>
+      </c>
+      <c r="C613" t="n">
+        <v>44.29</v>
+      </c>
+      <c r="D613" t="n">
+        <v>600</v>
+      </c>
+      <c r="E613" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="F613" t="n">
+        <v>600</v>
+      </c>
+      <c r="G613" t="n">
+        <v>30.1</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>13시</t>
+        </is>
+      </c>
+      <c r="C614" t="n">
+        <v>53.28</v>
+      </c>
+      <c r="D614" t="n">
+        <v>740</v>
+      </c>
+      <c r="E614" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="F614" t="n">
+        <v>740</v>
+      </c>
+      <c r="G614" t="n">
+        <v>31.3</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>14시</t>
+        </is>
+      </c>
+      <c r="C615" t="n">
+        <v>43.66</v>
+      </c>
+      <c r="D615" t="n">
+        <v>593</v>
+      </c>
+      <c r="E615" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="F615" t="n">
+        <v>593</v>
+      </c>
+      <c r="G615" t="n">
+        <v>30.9</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>15시</t>
+        </is>
+      </c>
+      <c r="C616" t="n">
+        <v>32.09</v>
+      </c>
+      <c r="D616" t="n">
+        <v>426</v>
+      </c>
+      <c r="E616" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="F616" t="n">
+        <v>426</v>
+      </c>
+      <c r="G616" t="n">
+        <v>30.9</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>16시</t>
+        </is>
+      </c>
+      <c r="C617" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="D617" t="n">
+        <v>407</v>
+      </c>
+      <c r="E617" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="F617" t="n">
+        <v>407</v>
+      </c>
+      <c r="G617" t="n">
+        <v>30.4</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>17시</t>
+        </is>
+      </c>
+      <c r="C618" t="n">
+        <v>26.96</v>
+      </c>
+      <c r="D618" t="n">
+        <v>353</v>
+      </c>
+      <c r="E618" t="n">
+        <v>30</v>
+      </c>
+      <c r="F618" t="n">
+        <v>353</v>
+      </c>
+      <c r="G618" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>18시</t>
+        </is>
+      </c>
+      <c r="C619" t="n">
+        <v>15.81</v>
+      </c>
+      <c r="D619" t="n">
+        <v>202</v>
+      </c>
+      <c r="E619" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="F619" t="n">
+        <v>202</v>
+      </c>
+      <c r="G619" t="n">
+        <v>28.9</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>19시</t>
+        </is>
+      </c>
+      <c r="C620" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="D620" t="n">
+        <v>71</v>
+      </c>
+      <c r="E620" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="F620" t="n">
+        <v>71</v>
+      </c>
+      <c r="G620" t="n">
+        <v>27.4</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>20시</t>
+        </is>
+      </c>
+      <c r="C621" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D621" t="n">
+        <v>3</v>
+      </c>
+      <c r="E621" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="F621" t="n">
+        <v>3</v>
+      </c>
+      <c r="G621" t="n">
+        <v>26.2</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>21시</t>
+        </is>
+      </c>
+      <c r="C622" t="n">
+        <v>0</v>
+      </c>
+      <c r="D622" t="n">
+        <v>0</v>
+      </c>
+      <c r="E622" t="n">
+        <v>25</v>
+      </c>
+      <c r="F622" t="n">
+        <v>0</v>
+      </c>
+      <c r="G622" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>22시</t>
+        </is>
+      </c>
+      <c r="C623" t="n">
+        <v>0</v>
+      </c>
+      <c r="D623" t="n">
+        <v>0</v>
+      </c>
+      <c r="E623" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="F623" t="n">
+        <v>0</v>
+      </c>
+      <c r="G623" t="n">
+        <v>24.2</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>23시</t>
+        </is>
+      </c>
+      <c r="C624" t="n">
+        <v>0</v>
+      </c>
+      <c r="D624" t="n">
+        <v>0</v>
+      </c>
+      <c r="E624" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F624" t="n">
+        <v>0</v>
+      </c>
+      <c r="G624" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>